<commit_message>
excel 2 coders ready
</commit_message>
<xml_diff>
--- a/outputs/originals/barcelona_samples_2015_2023_joined_results_20251103.xlsx
+++ b/outputs/originals/barcelona_samples_2015_2023_joined_results_20251103.xlsx
@@ -1015,7 +1015,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1104,6 +1104,18 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1113,6 +1125,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -13083,7 +13099,7 @@
         <f aca="false">ADD_evt!Q4</f>
         <v>1</v>
       </c>
-      <c r="K4" s="21" t="n">
+      <c r="K4" s="3" t="n">
         <f aca="false">ADD_evt!R4</f>
         <v>0</v>
       </c>
@@ -13095,7 +13111,7 @@
         <f aca="false">ADD_vgp!Q4</f>
         <v>1</v>
       </c>
-      <c r="N4" s="21" t="n">
+      <c r="N4" s="3" t="n">
         <f aca="false">ADD_vgp!R4</f>
         <v>0</v>
       </c>
@@ -13151,7 +13167,7 @@
         <f aca="false">ADD_evt!Q5</f>
         <v>0</v>
       </c>
-      <c r="K5" s="21" t="n">
+      <c r="K5" s="3" t="n">
         <f aca="false">ADD_evt!R5</f>
         <v>1</v>
       </c>
@@ -13163,7 +13179,7 @@
         <f aca="false">ADD_vgp!Q5</f>
         <v>0</v>
       </c>
-      <c r="N5" s="21" t="n">
+      <c r="N5" s="3" t="n">
         <f aca="false">ADD_vgp!R5</f>
         <v>1</v>
       </c>
@@ -13219,7 +13235,7 @@
         <f aca="false">ADD_evt!Q6</f>
         <v>0</v>
       </c>
-      <c r="K6" s="21" t="n">
+      <c r="K6" s="3" t="n">
         <f aca="false">ADD_evt!R6</f>
         <v>1</v>
       </c>
@@ -13231,7 +13247,7 @@
         <f aca="false">ADD_vgp!Q6</f>
         <v>0</v>
       </c>
-      <c r="N6" s="21" t="n">
+      <c r="N6" s="3" t="n">
         <f aca="false">ADD_vgp!R6</f>
         <v>1</v>
       </c>
@@ -13287,7 +13303,7 @@
         <f aca="false">ADD_evt!Q7</f>
         <v>0</v>
       </c>
-      <c r="K7" s="21" t="n">
+      <c r="K7" s="3" t="n">
         <f aca="false">ADD_evt!R7</f>
         <v>1</v>
       </c>
@@ -13299,7 +13315,7 @@
         <f aca="false">ADD_vgp!Q7</f>
         <v>0</v>
       </c>
-      <c r="N7" s="21" t="n">
+      <c r="N7" s="3" t="n">
         <f aca="false">ADD_vgp!R7</f>
         <v>1</v>
       </c>
@@ -13355,7 +13371,7 @@
         <f aca="false">ADD_evt!Q8</f>
         <v>0</v>
       </c>
-      <c r="K8" s="21" t="n">
+      <c r="K8" s="3" t="n">
         <f aca="false">ADD_evt!R8</f>
         <v>0</v>
       </c>
@@ -13367,7 +13383,7 @@
         <f aca="false">ADD_vgp!Q8</f>
         <v>0</v>
       </c>
-      <c r="N8" s="21" t="n">
+      <c r="N8" s="3" t="n">
         <f aca="false">ADD_vgp!R8</f>
         <v>0</v>
       </c>
@@ -13423,7 +13439,7 @@
         <f aca="false">ADD_evt!Q9</f>
         <v>0</v>
       </c>
-      <c r="K9" s="21" t="n">
+      <c r="K9" s="3" t="n">
         <f aca="false">ADD_evt!R9</f>
         <v>1</v>
       </c>
@@ -13435,7 +13451,7 @@
         <f aca="false">ADD_vgp!Q9</f>
         <v>0</v>
       </c>
-      <c r="N9" s="21" t="n">
+      <c r="N9" s="3" t="n">
         <f aca="false">ADD_vgp!R9</f>
         <v>1</v>
       </c>
@@ -13491,7 +13507,7 @@
         <f aca="false">ADD_evt!Q10</f>
         <v>0</v>
       </c>
-      <c r="K10" s="21" t="n">
+      <c r="K10" s="3" t="n">
         <f aca="false">ADD_evt!R10</f>
         <v>1</v>
       </c>
@@ -13503,7 +13519,7 @@
         <f aca="false">ADD_vgp!Q10</f>
         <v>0</v>
       </c>
-      <c r="N10" s="21" t="n">
+      <c r="N10" s="3" t="n">
         <f aca="false">ADD_vgp!R10</f>
         <v>1</v>
       </c>
@@ -13559,7 +13575,7 @@
         <f aca="false">ADD_evt!Q11</f>
         <v>0</v>
       </c>
-      <c r="K11" s="21" t="n">
+      <c r="K11" s="3" t="n">
         <f aca="false">ADD_evt!R11</f>
         <v>1</v>
       </c>
@@ -13571,7 +13587,7 @@
         <f aca="false">ADD_vgp!Q11</f>
         <v>0</v>
       </c>
-      <c r="N11" s="21" t="n">
+      <c r="N11" s="3" t="n">
         <f aca="false">ADD_vgp!R11</f>
         <v>1</v>
       </c>
@@ -13627,7 +13643,7 @@
         <f aca="false">ADD_evt!Q12</f>
         <v>NA</v>
       </c>
-      <c r="K12" s="21" t="e">
+      <c r="K12" s="3" t="e">
         <f aca="false">ADD_evt!R12</f>
         <v>#VALUE!</v>
       </c>
@@ -13639,7 +13655,7 @@
         <f aca="false">ADD_vgp!Q12</f>
         <v>1</v>
       </c>
-      <c r="N12" s="21" t="n">
+      <c r="N12" s="3" t="n">
         <f aca="false">ADD_vgp!R12</f>
         <v>0</v>
       </c>
@@ -13698,7 +13714,7 @@
         <f aca="false">ADD_evt!Q13</f>
         <v>1</v>
       </c>
-      <c r="K13" s="21" t="n">
+      <c r="K13" s="3" t="n">
         <f aca="false">ADD_evt!R13</f>
         <v>0</v>
       </c>
@@ -13710,7 +13726,7 @@
         <f aca="false">ADD_vgp!Q13</f>
         <v>1</v>
       </c>
-      <c r="N13" s="21" t="n">
+      <c r="N13" s="3" t="n">
         <f aca="false">ADD_vgp!R13</f>
         <v>0</v>
       </c>
@@ -13766,7 +13782,7 @@
         <f aca="false">ADD_evt!Q14</f>
         <v>1</v>
       </c>
-      <c r="K14" s="21" t="n">
+      <c r="K14" s="3" t="n">
         <f aca="false">ADD_evt!R14</f>
         <v>0</v>
       </c>
@@ -13778,7 +13794,7 @@
         <f aca="false">ADD_vgp!Q14</f>
         <v>1</v>
       </c>
-      <c r="N14" s="21" t="n">
+      <c r="N14" s="3" t="n">
         <f aca="false">ADD_vgp!R14</f>
         <v>0</v>
       </c>
@@ -13834,7 +13850,7 @@
         <f aca="false">ADD_evt!Q15</f>
         <v>0</v>
       </c>
-      <c r="K15" s="21" t="n">
+      <c r="K15" s="3" t="n">
         <f aca="false">ADD_evt!R15</f>
         <v>1</v>
       </c>
@@ -13846,7 +13862,7 @@
         <f aca="false">ADD_vgp!Q15</f>
         <v>0</v>
       </c>
-      <c r="N15" s="21" t="n">
+      <c r="N15" s="3" t="n">
         <f aca="false">ADD_vgp!R15</f>
         <v>1</v>
       </c>
@@ -13902,7 +13918,7 @@
         <f aca="false">ADD_evt!Q16</f>
         <v>0</v>
       </c>
-      <c r="K16" s="21" t="n">
+      <c r="K16" s="3" t="n">
         <f aca="false">ADD_evt!R16</f>
         <v>1</v>
       </c>
@@ -13914,7 +13930,7 @@
         <f aca="false">ADD_vgp!Q16</f>
         <v>0</v>
       </c>
-      <c r="N16" s="21" t="n">
+      <c r="N16" s="3" t="n">
         <f aca="false">ADD_vgp!R16</f>
         <v>1</v>
       </c>
@@ -13970,7 +13986,7 @@
         <f aca="false">ADD_evt!Q17</f>
         <v>0</v>
       </c>
-      <c r="K17" s="21" t="n">
+      <c r="K17" s="3" t="n">
         <f aca="false">ADD_evt!R17</f>
         <v>1</v>
       </c>
@@ -13982,7 +13998,7 @@
         <f aca="false">ADD_vgp!Q17</f>
         <v>0</v>
       </c>
-      <c r="N17" s="21" t="n">
+      <c r="N17" s="3" t="n">
         <f aca="false">ADD_vgp!R17</f>
         <v>1</v>
       </c>
@@ -14038,7 +14054,7 @@
         <f aca="false">ADD_evt!Q18</f>
         <v>0</v>
       </c>
-      <c r="K18" s="21" t="n">
+      <c r="K18" s="3" t="n">
         <f aca="false">ADD_evt!R18</f>
         <v>1</v>
       </c>
@@ -14050,7 +14066,7 @@
         <f aca="false">ADD_vgp!Q18</f>
         <v>0</v>
       </c>
-      <c r="N18" s="21" t="n">
+      <c r="N18" s="3" t="n">
         <f aca="false">ADD_vgp!R18</f>
         <v>1</v>
       </c>
@@ -14106,7 +14122,7 @@
         <f aca="false">ADD_evt!Q19</f>
         <v>0</v>
       </c>
-      <c r="K19" s="21" t="n">
+      <c r="K19" s="3" t="n">
         <f aca="false">ADD_evt!R19</f>
         <v>1</v>
       </c>
@@ -14118,7 +14134,7 @@
         <f aca="false">ADD_vgp!Q19</f>
         <v>0</v>
       </c>
-      <c r="N19" s="21" t="n">
+      <c r="N19" s="3" t="n">
         <f aca="false">ADD_vgp!R19</f>
         <v>1</v>
       </c>
@@ -14174,7 +14190,7 @@
         <f aca="false">ADD_evt!Q20</f>
         <v>0</v>
       </c>
-      <c r="K20" s="21" t="n">
+      <c r="K20" s="3" t="n">
         <f aca="false">ADD_evt!R20</f>
         <v>1</v>
       </c>
@@ -14186,7 +14202,7 @@
         <f aca="false">ADD_vgp!Q20</f>
         <v>0</v>
       </c>
-      <c r="N20" s="21" t="n">
+      <c r="N20" s="3" t="n">
         <f aca="false">ADD_vgp!R20</f>
         <v>1</v>
       </c>
@@ -14242,7 +14258,7 @@
         <f aca="false">ADD_evt!Q21</f>
         <v>0</v>
       </c>
-      <c r="K21" s="21" t="n">
+      <c r="K21" s="3" t="n">
         <f aca="false">ADD_evt!R21</f>
         <v>1</v>
       </c>
@@ -14254,7 +14270,7 @@
         <f aca="false">ADD_vgp!Q21</f>
         <v>0</v>
       </c>
-      <c r="N21" s="21" t="n">
+      <c r="N21" s="3" t="n">
         <f aca="false">ADD_vgp!R21</f>
         <v>1</v>
       </c>
@@ -14310,7 +14326,7 @@
         <f aca="false">ADD_evt!Q22</f>
         <v>0</v>
       </c>
-      <c r="K22" s="21" t="n">
+      <c r="K22" s="3" t="n">
         <f aca="false">ADD_evt!R22</f>
         <v>1</v>
       </c>
@@ -14322,7 +14338,7 @@
         <f aca="false">ADD_vgp!Q22</f>
         <v>0</v>
       </c>
-      <c r="N22" s="21" t="n">
+      <c r="N22" s="3" t="n">
         <f aca="false">ADD_vgp!R22</f>
         <v>1</v>
       </c>
@@ -14378,7 +14394,7 @@
         <f aca="false">ADD_evt!Q23</f>
         <v>1</v>
       </c>
-      <c r="K23" s="21" t="n">
+      <c r="K23" s="3" t="n">
         <f aca="false">ADD_evt!R23</f>
         <v>0</v>
       </c>
@@ -14390,7 +14406,7 @@
         <f aca="false">ADD_vgp!Q23</f>
         <v>1</v>
       </c>
-      <c r="N23" s="21" t="n">
+      <c r="N23" s="3" t="n">
         <f aca="false">ADD_vgp!R23</f>
         <v>0</v>
       </c>
@@ -14446,7 +14462,7 @@
         <f aca="false">ADD_evt!Q24</f>
         <v>1</v>
       </c>
-      <c r="K24" s="21" t="n">
+      <c r="K24" s="3" t="n">
         <f aca="false">ADD_evt!R24</f>
         <v>0</v>
       </c>
@@ -14458,7 +14474,7 @@
         <f aca="false">ADD_vgp!Q24</f>
         <v>1</v>
       </c>
-      <c r="N24" s="21" t="n">
+      <c r="N24" s="3" t="n">
         <f aca="false">ADD_vgp!R24</f>
         <v>0</v>
       </c>
@@ -14514,7 +14530,7 @@
         <f aca="false">ADD_evt!Q25</f>
         <v>0</v>
       </c>
-      <c r="K25" s="21" t="n">
+      <c r="K25" s="3" t="n">
         <f aca="false">ADD_evt!R25</f>
         <v>1</v>
       </c>
@@ -14526,7 +14542,7 @@
         <f aca="false">ADD_vgp!Q25</f>
         <v>0</v>
       </c>
-      <c r="N25" s="21" t="n">
+      <c r="N25" s="3" t="n">
         <f aca="false">ADD_vgp!R25</f>
         <v>1</v>
       </c>
@@ -14582,7 +14598,7 @@
         <f aca="false">ADD_evt!Q26</f>
         <v>0</v>
       </c>
-      <c r="K26" s="21" t="n">
+      <c r="K26" s="3" t="n">
         <f aca="false">ADD_evt!R26</f>
         <v>1</v>
       </c>
@@ -14594,7 +14610,7 @@
         <f aca="false">ADD_vgp!Q26</f>
         <v>0</v>
       </c>
-      <c r="N26" s="21" t="n">
+      <c r="N26" s="3" t="n">
         <f aca="false">ADD_vgp!R26</f>
         <v>1</v>
       </c>
@@ -14650,7 +14666,7 @@
         <f aca="false">ADD_evt!Q27</f>
         <v>NA</v>
       </c>
-      <c r="K27" s="21" t="e">
+      <c r="K27" s="3" t="e">
         <f aca="false">ADD_evt!R27</f>
         <v>#VALUE!</v>
       </c>
@@ -14662,7 +14678,7 @@
         <f aca="false">ADD_vgp!Q27</f>
         <v>0</v>
       </c>
-      <c r="N27" s="21" t="n">
+      <c r="N27" s="3" t="n">
         <f aca="false">ADD_vgp!R27</f>
         <v>1</v>
       </c>
@@ -14721,7 +14737,7 @@
         <f aca="false">ADD_evt!Q28</f>
         <v>0</v>
       </c>
-      <c r="K28" s="21" t="n">
+      <c r="K28" s="3" t="n">
         <f aca="false">ADD_evt!R28</f>
         <v>1</v>
       </c>
@@ -14733,7 +14749,7 @@
         <f aca="false">ADD_vgp!Q28</f>
         <v>0</v>
       </c>
-      <c r="N28" s="21" t="n">
+      <c r="N28" s="3" t="n">
         <f aca="false">ADD_vgp!R28</f>
         <v>1</v>
       </c>
@@ -14789,7 +14805,7 @@
         <f aca="false">ADD_evt!Q29</f>
         <v>0</v>
       </c>
-      <c r="K29" s="21" t="n">
+      <c r="K29" s="3" t="n">
         <f aca="false">ADD_evt!R29</f>
         <v>1</v>
       </c>
@@ -14801,7 +14817,7 @@
         <f aca="false">ADD_vgp!Q29</f>
         <v>0</v>
       </c>
-      <c r="N29" s="21" t="n">
+      <c r="N29" s="3" t="n">
         <f aca="false">ADD_vgp!R29</f>
         <v>1</v>
       </c>
@@ -14857,7 +14873,7 @@
         <f aca="false">ADD_evt!Q30</f>
         <v>0</v>
       </c>
-      <c r="K30" s="21" t="n">
+      <c r="K30" s="3" t="n">
         <f aca="false">ADD_evt!R30</f>
         <v>1</v>
       </c>
@@ -14869,7 +14885,7 @@
         <f aca="false">ADD_vgp!Q30</f>
         <v>0</v>
       </c>
-      <c r="N30" s="21" t="n">
+      <c r="N30" s="3" t="n">
         <f aca="false">ADD_vgp!R30</f>
         <v>1</v>
       </c>
@@ -14925,7 +14941,7 @@
         <f aca="false">ADD_evt!Q31</f>
         <v>0</v>
       </c>
-      <c r="K31" s="21" t="n">
+      <c r="K31" s="3" t="n">
         <f aca="false">ADD_evt!R31</f>
         <v>1</v>
       </c>
@@ -14937,7 +14953,7 @@
         <f aca="false">ADD_vgp!Q31</f>
         <v>0</v>
       </c>
-      <c r="N31" s="21" t="n">
+      <c r="N31" s="3" t="n">
         <f aca="false">ADD_vgp!R31</f>
         <v>1</v>
       </c>
@@ -14993,7 +15009,7 @@
         <f aca="false">ADD_evt!Q32</f>
         <v>0</v>
       </c>
-      <c r="K32" s="21" t="n">
+      <c r="K32" s="3" t="n">
         <f aca="false">ADD_evt!R32</f>
         <v>1</v>
       </c>
@@ -15005,7 +15021,7 @@
         <f aca="false">ADD_vgp!Q32</f>
         <v>0</v>
       </c>
-      <c r="N32" s="21" t="n">
+      <c r="N32" s="3" t="n">
         <f aca="false">ADD_vgp!R32</f>
         <v>1</v>
       </c>
@@ -15061,7 +15077,7 @@
         <f aca="false">ADD_evt!Q33</f>
         <v>NA</v>
       </c>
-      <c r="K33" s="21" t="e">
+      <c r="K33" s="3" t="e">
         <f aca="false">ADD_evt!R33</f>
         <v>#VALUE!</v>
       </c>
@@ -15073,7 +15089,7 @@
         <f aca="false">ADD_vgp!Q33</f>
         <v>1</v>
       </c>
-      <c r="N33" s="21" t="n">
+      <c r="N33" s="3" t="n">
         <f aca="false">ADD_vgp!R33</f>
         <v>0</v>
       </c>
@@ -15132,7 +15148,7 @@
         <f aca="false">ADD_evt!Q34</f>
         <v>0</v>
       </c>
-      <c r="K34" s="21" t="n">
+      <c r="K34" s="3" t="n">
         <f aca="false">ADD_evt!R34</f>
         <v>1</v>
       </c>
@@ -15144,7 +15160,7 @@
         <f aca="false">ADD_vgp!Q34</f>
         <v>0</v>
       </c>
-      <c r="N34" s="21" t="n">
+      <c r="N34" s="3" t="n">
         <f aca="false">ADD_vgp!R34</f>
         <v>1</v>
       </c>
@@ -15200,7 +15216,7 @@
         <f aca="false">ADD_evt!Q35</f>
         <v>0</v>
       </c>
-      <c r="K35" s="21" t="n">
+      <c r="K35" s="3" t="n">
         <f aca="false">ADD_evt!R35</f>
         <v>1</v>
       </c>
@@ -15212,7 +15228,7 @@
         <f aca="false">ADD_vgp!Q35</f>
         <v>0</v>
       </c>
-      <c r="N35" s="21" t="n">
+      <c r="N35" s="3" t="n">
         <f aca="false">ADD_vgp!R35</f>
         <v>1</v>
       </c>
@@ -15268,7 +15284,7 @@
         <f aca="false">ADD_evt!Q36</f>
         <v>0</v>
       </c>
-      <c r="K36" s="21" t="n">
+      <c r="K36" s="3" t="n">
         <f aca="false">ADD_evt!R36</f>
         <v>1</v>
       </c>
@@ -15280,7 +15296,7 @@
         <f aca="false">ADD_vgp!Q36</f>
         <v>0</v>
       </c>
-      <c r="N36" s="21" t="n">
+      <c r="N36" s="3" t="n">
         <f aca="false">ADD_vgp!R36</f>
         <v>1</v>
       </c>
@@ -15301,66 +15317,66 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="10" t="n">
+    <row r="37" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="22" t="n">
         <f aca="false">ADD_evt!A37</f>
         <v>35</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="D37" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="E37" s="1" t="n">
+      <c r="E37" s="23" t="n">
         <v>2.13075902951078</v>
       </c>
-      <c r="F37" s="1" t="n">
+      <c r="F37" s="23" t="n">
         <v>41.3750869481267</v>
       </c>
-      <c r="G37" s="1" t="s">
+      <c r="G37" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="H37" s="3" t="str">
+      <c r="H37" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.google.com/maps/@?api=1&amp;map_action=pano&amp;viewpoint=41.3750869481267,2.13075902951078","Open GSV")</f>
         <v>Open GSV</v>
       </c>
-      <c r="I37" s="3" t="str">
+      <c r="I37" s="24" t="str">
         <f aca="false">ADD_evt!P37</f>
         <v>0</v>
       </c>
-      <c r="J37" s="3" t="str">
+      <c r="J37" s="24" t="str">
         <f aca="false">ADD_evt!Q37</f>
         <v>0</v>
       </c>
-      <c r="K37" s="21" t="n">
+      <c r="K37" s="24" t="n">
         <f aca="false">ADD_evt!R37</f>
         <v>0</v>
       </c>
-      <c r="L37" s="3" t="str">
+      <c r="L37" s="24" t="str">
         <f aca="false">ADD_vgp!P37</f>
         <v>1</v>
       </c>
-      <c r="M37" s="3" t="str">
+      <c r="M37" s="24" t="str">
         <f aca="false">ADD_vgp!Q37</f>
         <v>1</v>
       </c>
-      <c r="N37" s="21" t="n">
+      <c r="N37" s="24" t="n">
         <f aca="false">ADD_vgp!R37</f>
         <v>0</v>
       </c>
-      <c r="O37" s="10" t="n">
+      <c r="O37" s="22" t="n">
         <f aca="false">IF(K37=N37,1,0)</f>
         <v>1</v>
       </c>
-      <c r="P37" s="1" t="n">
+      <c r="P37" s="23" t="n">
         <f aca="false">IF(O37=1,N(N37),"")</f>
         <v>0</v>
       </c>
-      <c r="R37" s="1" t="n">
+      <c r="R37" s="23" t="n">
         <f aca="false">IF(
    OR(ISERROR(P37), ISERROR(Q37), P37="NA", Q37="NA"),
    "NA",
@@ -15369,66 +15385,66 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="10" t="n">
+    <row r="38" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="22" t="n">
         <f aca="false">ADD_evt!A38</f>
         <v>36</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C38" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D38" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="E38" s="1" t="n">
+      <c r="E38" s="23" t="n">
         <v>2.13118777902404</v>
       </c>
-      <c r="F38" s="1" t="n">
+      <c r="F38" s="23" t="n">
         <v>41.3738399462803</v>
       </c>
-      <c r="G38" s="1" t="s">
+      <c r="G38" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="H38" s="3" t="str">
+      <c r="H38" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.google.com/maps/@?api=1&amp;map_action=pano&amp;viewpoint=41.3738399462803,2.13118777902404","Open GSV")</f>
         <v>Open GSV</v>
       </c>
-      <c r="I38" s="3" t="str">
+      <c r="I38" s="24" t="str">
         <f aca="false">ADD_evt!P38</f>
         <v>0</v>
       </c>
-      <c r="J38" s="3" t="str">
+      <c r="J38" s="24" t="str">
         <f aca="false">ADD_evt!Q38</f>
         <v>0</v>
       </c>
-      <c r="K38" s="21" t="n">
+      <c r="K38" s="24" t="n">
         <f aca="false">ADD_evt!R38</f>
         <v>0</v>
       </c>
-      <c r="L38" s="3" t="str">
+      <c r="L38" s="24" t="str">
         <f aca="false">ADD_vgp!P38</f>
         <v>1</v>
       </c>
-      <c r="M38" s="3" t="str">
+      <c r="M38" s="24" t="str">
         <f aca="false">ADD_vgp!Q38</f>
         <v>1</v>
       </c>
-      <c r="N38" s="21" t="n">
+      <c r="N38" s="24" t="n">
         <f aca="false">ADD_vgp!R38</f>
         <v>0</v>
       </c>
-      <c r="O38" s="10" t="n">
+      <c r="O38" s="22" t="n">
         <f aca="false">IF(K38=N38,1,0)</f>
         <v>1</v>
       </c>
-      <c r="P38" s="1" t="n">
+      <c r="P38" s="23" t="n">
         <f aca="false">IF(O38=1,N(N38),"")</f>
         <v>0</v>
       </c>
-      <c r="R38" s="1" t="n">
+      <c r="R38" s="23" t="n">
         <f aca="false">IF(
    OR(ISERROR(P38), ISERROR(Q38), P38="NA", Q38="NA"),
    "NA",
@@ -15437,69 +15453,69 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="10" t="n">
+    <row r="39" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="22" t="n">
         <f aca="false">ADD_evt!A39</f>
         <v>37</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C39" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="D39" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="E39" s="1" t="n">
+      <c r="E39" s="23" t="n">
         <v>2.17976081270431</v>
       </c>
-      <c r="F39" s="1" t="n">
+      <c r="F39" s="23" t="n">
         <v>41.4118804921771</v>
       </c>
-      <c r="G39" s="1" t="s">
+      <c r="G39" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="H39" s="3" t="str">
+      <c r="H39" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.google.com/maps/@?api=1&amp;map_action=pano&amp;viewpoint=41.4118804921771,2.17976081270431","Open GSV")</f>
         <v>Open GSV</v>
       </c>
-      <c r="I39" s="3" t="str">
+      <c r="I39" s="24" t="str">
         <f aca="false">ADD_evt!P39</f>
         <v>1</v>
       </c>
-      <c r="J39" s="3" t="str">
+      <c r="J39" s="24" t="str">
         <f aca="false">ADD_evt!Q39</f>
         <v>0</v>
       </c>
-      <c r="K39" s="21" t="n">
+      <c r="K39" s="24" t="n">
         <f aca="false">ADD_evt!R39</f>
         <v>1</v>
       </c>
-      <c r="L39" s="3" t="str">
+      <c r="L39" s="24" t="str">
         <f aca="false">ADD_vgp!P39</f>
         <v>0</v>
       </c>
-      <c r="M39" s="3" t="str">
+      <c r="M39" s="24" t="str">
         <f aca="false">ADD_vgp!Q39</f>
         <v>0</v>
       </c>
-      <c r="N39" s="21" t="n">
+      <c r="N39" s="24" t="n">
         <f aca="false">ADD_vgp!R39</f>
         <v>0</v>
       </c>
-      <c r="O39" s="10" t="n">
+      <c r="O39" s="22" t="n">
         <f aca="false">IF(K39=N39,1,0)</f>
         <v>0</v>
       </c>
-      <c r="P39" s="1" t="str">
+      <c r="P39" s="23" t="str">
         <f aca="false">IF(O39=1,N(N39),"")</f>
         <v/>
       </c>
-      <c r="Q39" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="R39" s="1" t="n">
+      <c r="Q39" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="R39" s="23" t="n">
         <f aca="false">IF(
    OR(ISERROR(P39), ISERROR(Q39), P39="NA", Q39="NA"),
    "NA",
@@ -15507,70 +15523,70 @@
 )</f>
         <v>1</v>
       </c>
-      <c r="S39" s="1" t="s">
+      <c r="S39" s="23" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="40" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="10" t="n">
+    <row r="40" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="22" t="n">
         <f aca="false">ADD_evt!A40</f>
         <v>38</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D40" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="E40" s="1" t="n">
+      <c r="E40" s="23" t="n">
         <v>2.180890772398</v>
       </c>
-      <c r="F40" s="1" t="n">
+      <c r="F40" s="23" t="n">
         <v>41.4127447371871</v>
       </c>
-      <c r="G40" s="1" t="s">
+      <c r="G40" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="H40" s="3" t="str">
+      <c r="H40" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.google.com/maps/@?api=1&amp;map_action=pano&amp;viewpoint=41.4127447371871,2.180890772398","Open GSV")</f>
         <v>Open GSV</v>
       </c>
-      <c r="I40" s="3" t="str">
+      <c r="I40" s="24" t="str">
         <f aca="false">ADD_evt!P40</f>
         <v>0</v>
       </c>
-      <c r="J40" s="3" t="str">
+      <c r="J40" s="24" t="str">
         <f aca="false">ADD_evt!Q40</f>
         <v>0</v>
       </c>
-      <c r="K40" s="21" t="n">
+      <c r="K40" s="24" t="n">
         <f aca="false">ADD_evt!R40</f>
         <v>0</v>
       </c>
-      <c r="L40" s="3" t="str">
+      <c r="L40" s="24" t="str">
         <f aca="false">ADD_vgp!P40</f>
         <v>0</v>
       </c>
-      <c r="M40" s="3" t="str">
+      <c r="M40" s="24" t="str">
         <f aca="false">ADD_vgp!Q40</f>
         <v>0</v>
       </c>
-      <c r="N40" s="21" t="n">
+      <c r="N40" s="24" t="n">
         <f aca="false">ADD_vgp!R40</f>
         <v>0</v>
       </c>
-      <c r="O40" s="10" t="n">
+      <c r="O40" s="22" t="n">
         <f aca="false">IF(K40=N40,1,0)</f>
         <v>1</v>
       </c>
-      <c r="P40" s="1" t="n">
+      <c r="P40" s="23" t="n">
         <f aca="false">IF(O40=1,N(N40),"")</f>
         <v>0</v>
       </c>
-      <c r="R40" s="1" t="n">
+      <c r="R40" s="23" t="n">
         <f aca="false">IF(
    OR(ISERROR(P40), ISERROR(Q40), P40="NA", Q40="NA"),
    "NA",
@@ -15614,7 +15630,7 @@
         <f aca="false">ADD_evt!Q41</f>
         <v>0</v>
       </c>
-      <c r="K41" s="21" t="n">
+      <c r="K41" s="3" t="n">
         <f aca="false">ADD_evt!R41</f>
         <v>1</v>
       </c>
@@ -15626,7 +15642,7 @@
         <f aca="false">ADD_vgp!Q41</f>
         <v>0</v>
       </c>
-      <c r="N41" s="21" t="n">
+      <c r="N41" s="3" t="n">
         <f aca="false">ADD_vgp!R41</f>
         <v>1</v>
       </c>
@@ -15682,7 +15698,7 @@
         <f aca="false">ADD_evt!Q42</f>
         <v>0</v>
       </c>
-      <c r="K42" s="21" t="n">
+      <c r="K42" s="3" t="n">
         <f aca="false">ADD_evt!R42</f>
         <v>1</v>
       </c>
@@ -15694,7 +15710,7 @@
         <f aca="false">ADD_vgp!Q42</f>
         <v>0</v>
       </c>
-      <c r="N42" s="21" t="n">
+      <c r="N42" s="3" t="n">
         <f aca="false">ADD_vgp!R42</f>
         <v>1</v>
       </c>
@@ -15750,7 +15766,7 @@
         <f aca="false">ADD_evt!Q43</f>
         <v>0</v>
       </c>
-      <c r="K43" s="21" t="n">
+      <c r="K43" s="3" t="n">
         <f aca="false">ADD_evt!R43</f>
         <v>1</v>
       </c>
@@ -15762,7 +15778,7 @@
         <f aca="false">ADD_vgp!Q43</f>
         <v>0</v>
       </c>
-      <c r="N43" s="21" t="n">
+      <c r="N43" s="3" t="n">
         <f aca="false">ADD_vgp!R43</f>
         <v>1</v>
       </c>
@@ -15818,7 +15834,7 @@
         <f aca="false">ADD_evt!Q44</f>
         <v>0</v>
       </c>
-      <c r="K44" s="21" t="n">
+      <c r="K44" s="3" t="n">
         <f aca="false">ADD_evt!R44</f>
         <v>1</v>
       </c>
@@ -15830,7 +15846,7 @@
         <f aca="false">ADD_vgp!Q44</f>
         <v>0</v>
       </c>
-      <c r="N44" s="21" t="n">
+      <c r="N44" s="3" t="n">
         <f aca="false">ADD_vgp!R44</f>
         <v>1</v>
       </c>
@@ -15887,7 +15903,7 @@
         <f aca="false">ADD_evt!Q45</f>
         <v>0</v>
       </c>
-      <c r="K45" s="21" t="n">
+      <c r="K45" s="3" t="n">
         <f aca="false">ADD_evt!R45</f>
         <v>1</v>
       </c>
@@ -15899,7 +15915,7 @@
         <f aca="false">ADD_vgp!Q45</f>
         <v>0</v>
       </c>
-      <c r="N45" s="21" t="n">
+      <c r="N45" s="3" t="n">
         <f aca="false">ADD_vgp!R45</f>
         <v>1</v>
       </c>
@@ -15955,7 +15971,7 @@
         <f aca="false">ADD_evt!Q46</f>
         <v>0</v>
       </c>
-      <c r="K46" s="21" t="n">
+      <c r="K46" s="3" t="n">
         <f aca="false">ADD_evt!R46</f>
         <v>1</v>
       </c>
@@ -15967,7 +15983,7 @@
         <f aca="false">ADD_vgp!Q46</f>
         <v>0</v>
       </c>
-      <c r="N46" s="21" t="n">
+      <c r="N46" s="3" t="n">
         <f aca="false">ADD_vgp!R46</f>
         <v>1</v>
       </c>
@@ -16023,7 +16039,7 @@
         <f aca="false">ADD_evt!Q47</f>
         <v>0</v>
       </c>
-      <c r="K47" s="21" t="n">
+      <c r="K47" s="3" t="n">
         <f aca="false">ADD_evt!R47</f>
         <v>1</v>
       </c>
@@ -16035,7 +16051,7 @@
         <f aca="false">ADD_vgp!Q47</f>
         <v>0</v>
       </c>
-      <c r="N47" s="21" t="n">
+      <c r="N47" s="3" t="n">
         <f aca="false">ADD_vgp!R47</f>
         <v>1</v>
       </c>
@@ -16091,7 +16107,7 @@
         <f aca="false">ADD_evt!Q48</f>
         <v>NA</v>
       </c>
-      <c r="K48" s="21" t="e">
+      <c r="K48" s="3" t="e">
         <f aca="false">ADD_evt!R48</f>
         <v>#VALUE!</v>
       </c>
@@ -16103,7 +16119,7 @@
         <f aca="false">ADD_vgp!Q48</f>
         <v>1</v>
       </c>
-      <c r="N48" s="21" t="n">
+      <c r="N48" s="3" t="n">
         <f aca="false">ADD_vgp!R48</f>
         <v>0</v>
       </c>
@@ -16165,7 +16181,7 @@
         <f aca="false">ADD_evt!Q49</f>
         <v>0</v>
       </c>
-      <c r="K49" s="21" t="n">
+      <c r="K49" s="3" t="n">
         <f aca="false">ADD_evt!R49</f>
         <v>1</v>
       </c>
@@ -16177,7 +16193,7 @@
         <f aca="false">ADD_vgp!Q49</f>
         <v>0</v>
       </c>
-      <c r="N49" s="21" t="n">
+      <c r="N49" s="3" t="n">
         <f aca="false">ADD_vgp!R49</f>
         <v>0</v>
       </c>
@@ -16239,7 +16255,7 @@
         <f aca="false">ADD_evt!Q50</f>
         <v>0</v>
       </c>
-      <c r="K50" s="21" t="n">
+      <c r="K50" s="3" t="n">
         <f aca="false">ADD_evt!R50</f>
         <v>1</v>
       </c>
@@ -16251,7 +16267,7 @@
         <f aca="false">ADD_vgp!Q50</f>
         <v>0</v>
       </c>
-      <c r="N50" s="21" t="n">
+      <c r="N50" s="3" t="n">
         <f aca="false">ADD_vgp!R50</f>
         <v>0</v>
       </c>
@@ -16284,20 +16300,18 @@
         <v>41</v>
       </c>
       <c r="P51" s="12"/>
-      <c r="Q51" s="0"/>
       <c r="R51" s="12" t="n">
         <f aca="false">COUNTIFS(R3:R50,1)</f>
         <v>34</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O52" s="22" t="n">
+      <c r="O52" s="25" t="n">
         <f aca="false">COUNTIFS(O3:O50,1) / (COUNTIFS(O3:O50,1) + COUNTIFS(O3:O50,0))</f>
         <v>0.931818181818182</v>
       </c>
-      <c r="P52" s="22"/>
-      <c r="Q52" s="0"/>
-      <c r="R52" s="23" t="n">
+      <c r="P52" s="25"/>
+      <c r="R52" s="26" t="n">
         <f aca="false">COUNTIFS(R3:R50,1) / (COUNTIFS(R3:R50,1) + COUNTIFS(R3:R50,0))</f>
         <v>0.772727272727273</v>
       </c>
@@ -16450,7 +16464,7 @@
         <f aca="false">IF(O3=1, N(N3), "")</f>
         <v>0</v>
       </c>
-      <c r="Q3" s="24"/>
+      <c r="Q3" s="27"/>
       <c r="R3" s="1" t="n">
         <f aca="false">IF(
    OR(ISERROR(P3), ISERROR(Q3), P3="NA", Q3="NA"),
@@ -16495,7 +16509,7 @@
         <f aca="false">REMOVE_evt!Q4</f>
         <v>1</v>
       </c>
-      <c r="K4" s="21" t="n">
+      <c r="K4" s="3" t="n">
         <f aca="false">REMOVE_evt!R4</f>
         <v>0</v>
       </c>
@@ -16507,7 +16521,7 @@
         <f aca="false">REMOVE_vgp!Q4</f>
         <v>1</v>
       </c>
-      <c r="N4" s="21" t="n">
+      <c r="N4" s="3" t="n">
         <f aca="false">REMOVE_vgp!R4</f>
         <v>0</v>
       </c>
@@ -16519,7 +16533,7 @@
         <f aca="false">IF(O4=1, N(N4), "")</f>
         <v>0</v>
       </c>
-      <c r="Q4" s="24"/>
+      <c r="Q4" s="27"/>
       <c r="R4" s="1" t="n">
         <f aca="false">IF(
    OR(ISERROR(P4), ISERROR(Q4), P4="NA", Q4="NA"),
@@ -16564,7 +16578,7 @@
         <f aca="false">REMOVE_evt!Q5</f>
         <v>0</v>
       </c>
-      <c r="K5" s="21" t="n">
+      <c r="K5" s="3" t="n">
         <f aca="false">REMOVE_evt!R5</f>
         <v>0</v>
       </c>
@@ -16576,7 +16590,7 @@
         <f aca="false">REMOVE_vgp!Q5</f>
         <v>0</v>
       </c>
-      <c r="N5" s="21" t="n">
+      <c r="N5" s="3" t="n">
         <f aca="false">REMOVE_vgp!R5</f>
         <v>0</v>
       </c>
@@ -16588,7 +16602,7 @@
         <f aca="false">IF(O5=1, N(N5), "")</f>
         <v>0</v>
       </c>
-      <c r="Q5" s="24"/>
+      <c r="Q5" s="27"/>
       <c r="R5" s="1" t="n">
         <f aca="false">IF(
    OR(ISERROR(P5), ISERROR(Q5), P5="NA", Q5="NA"),
@@ -16633,7 +16647,7 @@
         <f aca="false">REMOVE_evt!Q6</f>
         <v>0</v>
       </c>
-      <c r="K6" s="21" t="n">
+      <c r="K6" s="3" t="n">
         <f aca="false">REMOVE_evt!R6</f>
         <v>0</v>
       </c>
@@ -16645,7 +16659,7 @@
         <f aca="false">REMOVE_vgp!Q6</f>
         <v>0</v>
       </c>
-      <c r="N6" s="21" t="n">
+      <c r="N6" s="3" t="n">
         <f aca="false">REMOVE_vgp!R6</f>
         <v>0</v>
       </c>
@@ -16657,7 +16671,7 @@
         <f aca="false">IF(O6=1, N(N6), "")</f>
         <v>0</v>
       </c>
-      <c r="Q6" s="24"/>
+      <c r="Q6" s="27"/>
       <c r="R6" s="1" t="n">
         <f aca="false">IF(
    OR(ISERROR(P6), ISERROR(Q6), P6="NA", Q6="NA"),
@@ -16667,67 +16681,67 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="n">
+    <row r="7" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="22" t="n">
         <f aca="false">REMOVE_evt!A7</f>
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="23" t="n">
         <v>2.17443553665477</v>
       </c>
-      <c r="F7" s="1" t="n">
+      <c r="F7" s="23" t="n">
         <v>41.4302401188698</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="H7" s="3" t="str">
+      <c r="H7" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.google.com/maps/@?api=1&amp;map_action=pano&amp;viewpoint=41.4302401188698,2.17443553665477","Open GSV")</f>
         <v>Open GSV</v>
       </c>
-      <c r="I7" s="3" t="str">
+      <c r="I7" s="24" t="str">
         <f aca="false">REMOVE_evt!P7</f>
         <v>0</v>
       </c>
-      <c r="J7" s="3" t="str">
+      <c r="J7" s="24" t="str">
         <f aca="false">REMOVE_evt!Q7</f>
         <v>0</v>
       </c>
-      <c r="K7" s="21" t="n">
+      <c r="K7" s="24" t="n">
         <f aca="false">REMOVE_evt!R7</f>
         <v>0</v>
       </c>
-      <c r="L7" s="3" t="str">
+      <c r="L7" s="24" t="str">
         <f aca="false">REMOVE_vgp!P7</f>
         <v>1</v>
       </c>
-      <c r="M7" s="3" t="str">
+      <c r="M7" s="24" t="str">
         <f aca="false">REMOVE_vgp!Q7</f>
         <v>1</v>
       </c>
-      <c r="N7" s="21" t="n">
+      <c r="N7" s="24" t="n">
         <f aca="false">REMOVE_vgp!R7</f>
         <v>0</v>
       </c>
-      <c r="O7" s="10" t="n">
+      <c r="O7" s="22" t="n">
         <f aca="false">IF(K7=N7,1,0)</f>
         <v>1</v>
       </c>
-      <c r="P7" s="1" t="n">
+      <c r="P7" s="23" t="n">
         <f aca="false">IF(O7=1, N(N7), "")</f>
         <v>0</v>
       </c>
-      <c r="Q7" s="24"/>
-      <c r="R7" s="1" t="n">
+      <c r="Q7" s="28"/>
+      <c r="R7" s="23" t="n">
         <f aca="false">IF(
    OR(ISERROR(P7), ISERROR(Q7), P7="NA", Q7="NA"),
    "NA",
@@ -16771,7 +16785,7 @@
         <f aca="false">REMOVE_evt!Q8</f>
         <v>1</v>
       </c>
-      <c r="K8" s="21" t="n">
+      <c r="K8" s="3" t="n">
         <f aca="false">REMOVE_evt!R8</f>
         <v>1</v>
       </c>
@@ -16783,7 +16797,7 @@
         <f aca="false">REMOVE_vgp!Q8</f>
         <v>1</v>
       </c>
-      <c r="N8" s="21" t="n">
+      <c r="N8" s="3" t="n">
         <f aca="false">REMOVE_vgp!R8</f>
         <v>1</v>
       </c>
@@ -16795,7 +16809,7 @@
         <f aca="false">IF(O8=1, N(N8), "")</f>
         <v>1</v>
       </c>
-      <c r="Q8" s="24"/>
+      <c r="Q8" s="27"/>
       <c r="R8" s="1" t="n">
         <f aca="false">IF(
    OR(ISERROR(P8), ISERROR(Q8), P8="NA", Q8="NA"),
@@ -16840,7 +16854,7 @@
         <f aca="false">REMOVE_evt!Q9</f>
         <v>NA</v>
       </c>
-      <c r="K9" s="21" t="e">
+      <c r="K9" s="3" t="e">
         <f aca="false">REMOVE_evt!R9</f>
         <v>#VALUE!</v>
       </c>
@@ -16852,7 +16866,7 @@
         <f aca="false">REMOVE_vgp!Q9</f>
         <v>1</v>
       </c>
-      <c r="N9" s="21" t="n">
+      <c r="N9" s="3" t="n">
         <f aca="false">REMOVE_vgp!R9</f>
         <v>1</v>
       </c>
@@ -16864,7 +16878,7 @@
         <f aca="false">IF(O9=1, N(N9), "")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="Q9" s="24"/>
+      <c r="Q9" s="27"/>
       <c r="R9" s="1" t="e">
         <f aca="false">IF(
    OR(ISERROR(P9), ISERROR(Q9), P9="NA", Q9="NA"),
@@ -16912,7 +16926,7 @@
         <f aca="false">REMOVE_evt!Q10</f>
         <v>1</v>
       </c>
-      <c r="K10" s="21" t="n">
+      <c r="K10" s="3" t="n">
         <f aca="false">REMOVE_evt!R10</f>
         <v>1</v>
       </c>
@@ -16924,7 +16938,7 @@
         <f aca="false">REMOVE_vgp!Q10</f>
         <v>1</v>
       </c>
-      <c r="N10" s="21" t="n">
+      <c r="N10" s="3" t="n">
         <f aca="false">REMOVE_vgp!R10</f>
         <v>1</v>
       </c>
@@ -16936,7 +16950,7 @@
         <f aca="false">IF(O10=1, N(N10), "")</f>
         <v>1</v>
       </c>
-      <c r="Q10" s="24"/>
+      <c r="Q10" s="27"/>
       <c r="R10" s="1" t="n">
         <f aca="false">IF(
    OR(ISERROR(P10), ISERROR(Q10), P10="NA", Q10="NA"),
@@ -16989,13 +17003,13 @@
       <c r="L12" s="10"/>
       <c r="M12" s="10"/>
       <c r="N12" s="10"/>
-      <c r="O12" s="22" t="n">
+      <c r="O12" s="25" t="n">
         <f aca="false">COUNTIFS(O3:O10,1) / (COUNTIFS(O3:O10,1) + COUNTIFS(O3:O10,0))</f>
         <v>1</v>
       </c>
-      <c r="P12" s="22"/>
-      <c r="Q12" s="22"/>
-      <c r="R12" s="23" t="n">
+      <c r="P12" s="25"/>
+      <c r="Q12" s="25"/>
+      <c r="R12" s="26" t="n">
         <f aca="false">COUNTIFS(R3:R10,1) / (COUNTIFS(R3:R10,1) + COUNTIFS(R3:R10,0))</f>
         <v>0.285714285714286</v>
       </c>
@@ -17050,14 +17064,11 @@
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="7" min="7" style="1" width="12.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="9" style="1" width="15.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="12.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="12.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="1" width="12.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="13.81"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q1" s="0"/>
-    </row>
+    <row r="1" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="2" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
         <v>2</v>
@@ -18542,66 +18553,66 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="n">
+    <row r="24" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="22" t="n">
         <f aca="false">NONCI_evt!A24</f>
         <v>22</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="23" t="s">
         <v>164</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D24" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="E24" s="23" t="n">
         <v>2.17554070368043</v>
       </c>
-      <c r="F24" s="1" t="n">
+      <c r="F24" s="23" t="n">
         <v>41.4280696452023</v>
       </c>
-      <c r="G24" s="1" t="s">
+      <c r="G24" s="23" t="s">
         <v>194</v>
       </c>
-      <c r="H24" s="3" t="str">
+      <c r="H24" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.google.com/maps/@?api=1&amp;map_action=pano&amp;viewpoint=41.4280696452023,2.17554070368043","Open GSV")</f>
         <v>Open GSV</v>
       </c>
-      <c r="I24" s="3" t="str">
+      <c r="I24" s="24" t="str">
         <f aca="false">NONCI_evt!P24</f>
         <v>0</v>
       </c>
-      <c r="J24" s="3" t="str">
+      <c r="J24" s="24" t="str">
         <f aca="false">NONCI_evt!Q24</f>
         <v>0</v>
       </c>
-      <c r="K24" s="3" t="n">
+      <c r="K24" s="24" t="n">
         <f aca="false">NONCI_evt!R24</f>
         <v>1</v>
       </c>
-      <c r="L24" s="3" t="str">
+      <c r="L24" s="24" t="str">
         <f aca="false">NONCI_vgp!P24</f>
         <v>1</v>
       </c>
-      <c r="M24" s="3" t="str">
+      <c r="M24" s="24" t="str">
         <f aca="false">NONCI_vgp!Q24</f>
         <v>1</v>
       </c>
-      <c r="N24" s="3" t="n">
+      <c r="N24" s="24" t="n">
         <f aca="false">NONCI_vgp!R24</f>
         <v>0</v>
       </c>
-      <c r="O24" s="10" t="n">
+      <c r="O24" s="22" t="n">
         <f aca="false">IF(K24=N24,1,0)</f>
         <v>0</v>
       </c>
-      <c r="P24" s="1" t="str">
+      <c r="P24" s="23" t="str">
         <f aca="false">IF(O24=1,N(N24),"")</f>
         <v/>
       </c>
-      <c r="R24" s="1" t="n">
+      <c r="R24" s="23" t="n">
         <f aca="false">IF(
    OR(ISERROR(P24), ISERROR(Q24), P24="NA", Q24="NA"),
    "NA",
@@ -18609,7 +18620,7 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="S24" s="1" t="s">
+      <c r="S24" s="23" t="s">
         <v>262</v>
       </c>
     </row>
@@ -20440,7 +20451,6 @@
         <f aca="false">IF(O51=1,N(N51),"")</f>
         <v>1</v>
       </c>
-      <c r="Q51" s="1"/>
       <c r="R51" s="1" t="n">
         <f aca="false">IF(
    OR(ISERROR(P51), ISERROR(Q51), P51="NA", Q51="NA"),
@@ -20494,12 +20504,12 @@
       <c r="L53" s="10"/>
       <c r="M53" s="10"/>
       <c r="N53" s="10"/>
-      <c r="O53" s="22" t="n">
+      <c r="O53" s="25" t="n">
         <f aca="false">COUNTIFS(O3:O51,1) / (COUNTIFS(O3:O51,1) + COUNTIFS(O3:O51,0))</f>
         <v>0.977272727272727</v>
       </c>
-      <c r="P53" s="22"/>
-      <c r="R53" s="23" t="n">
+      <c r="P53" s="25"/>
+      <c r="R53" s="26" t="n">
         <f aca="false">COUNTIFS(R3:R51,1) / (COUNTIFS(R3:R51,1) + COUNTIFS(R3:R51,0))</f>
         <v>0.954545454545455</v>
       </c>

</xml_diff>